<commit_message>
feat: update process hierarchy register to 6 node groups & 31 processes (20260905 BL), add Version_Control.md, and update README.md
</commit_message>
<xml_diff>
--- a/SAP_B1_Process_Design_Matrix.xlsx
+++ b/SAP_B1_Process_Design_Matrix.xlsx
@@ -1445,7 +1445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2745,7 +2745,7 @@
     <row r="31" ht="32" customHeight="1">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>2.5 [SNG-RECON]</t>
+          <t>2.5 [SNG-RECONCILIATION]</t>
         </is>
       </c>
       <c r="B31" s="12" t="inlineStr">
@@ -2792,7 +2792,7 @@
     <row r="32" ht="32" customHeight="1">
       <c r="A32" s="16" t="inlineStr">
         <is>
-          <t>2.5 [SNG-RECON]</t>
+          <t>2.5 [SNG-RECONCILIATION]</t>
         </is>
       </c>
       <c r="B32" s="16" t="inlineStr">
@@ -2833,6 +2833,147 @@
       <c r="I32" s="19" t="inlineStr">
         <is>
           <t>OIPF, IPF1, IPF2, OPCH, OJDT (200050)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="32" customHeight="1">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>2.5 [SNG-RECONCILIATION]</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>2.5.3</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>Group Report Reconciliation</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>new_b1 + old_b1</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>All Hubs</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>Consolidated Ledgers</t>
+        </is>
+      </c>
+      <c r="G33" s="14" t="inlineStr">
+        <is>
+          <t>Group Financial Statements</t>
+        </is>
+      </c>
+      <c r="H33" s="13" t="inlineStr">
+        <is>
+          <t>Intercompany elimination, group inventory valuation consolidation, and multi-entity profit reporting</t>
+        </is>
+      </c>
+      <c r="I33" s="15" t="inlineStr">
+        <is>
+          <t>OJDT, JDT1, OACT, Group Balance Sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>2.6 [MD-MAINTENANCE]</t>
+        </is>
+      </c>
+      <c r="B34" s="16" t="inlineStr">
+        <is>
+          <t>2.6.1</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>SAP B1 Inventory Item Master Maintenance</t>
+        </is>
+      </c>
+      <c r="D34" s="18" t="inlineStr">
+        <is>
+          <t>new_b1 + old_b1</t>
+        </is>
+      </c>
+      <c r="E34" s="18" t="inlineStr">
+        <is>
+          <t>Master Setup</t>
+        </is>
+      </c>
+      <c r="F34" s="18" t="inlineStr">
+        <is>
+          <t>Warehouse Bins</t>
+        </is>
+      </c>
+      <c r="G34" s="18" t="inlineStr">
+        <is>
+          <t>Item Master Records</t>
+        </is>
+      </c>
+      <c r="H34" s="17" t="inlineStr">
+        <is>
+          <t>Item Code creation, valuation method setup (OITM vs OITW), purchasing/sales UoM, and barcode cataloging</t>
+        </is>
+      </c>
+      <c r="I34" s="19" t="inlineStr">
+        <is>
+          <t>OITM, OITW, ITM1, OPLN, OWHS, OBIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="32" customHeight="1">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>2.6 [MD-MAINTENANCE]</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>2.6.2</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>SAP B1 Business Partner Master Maintenance</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>new_b1 + old_b1</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>Master Setup</t>
+        </is>
+      </c>
+      <c r="F35" s="14" t="inlineStr">
+        <is>
+          <t>Commercial Ledger</t>
+        </is>
+      </c>
+      <c r="G35" s="14" t="inlineStr">
+        <is>
+          <t>BP Master Records</t>
+        </is>
+      </c>
+      <c r="H35" s="13" t="inlineStr">
+        <is>
+          <t>Vendor/Customer setup (OCRD/CRD1), currency assignment (USD/AUD/NZD/GBP), payment terms (OCTG), and tax group mapping</t>
+        </is>
+      </c>
+      <c r="I35" s="15" t="inlineStr">
+        <is>
+          <t>OCRD, CRD1, OCPR, OCRG, OCTG, OSTC</t>
         </is>
       </c>
     </row>

</xml_diff>